<commit_message>
Update NextGen PMO saved work and dashboard assets
</commit_message>
<xml_diff>
--- a/NG Scheduling.xlsx
+++ b/NG Scheduling.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://my.wal-mart.com/personal/k0m0eg1_homeoffice_wal-mart_com/Documents/Desktop/Code Puppy Saved Work/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1895" documentId="8_{3CD9A91E-A1DC-493E-B251-6A7E654DFCDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7F43286D-E8F8-4A01-B963-46D5338EDD9C}"/>
+  <xr:revisionPtr revIDLastSave="1926" documentId="8_{3CD9A91E-A1DC-493E-B251-6A7E654DFCDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C4765751-D525-45D9-B898-F8D4FD33921A}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="90" yWindow="90" windowWidth="23028" windowHeight="13668" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="2100" yWindow="2295" windowWidth="38220" windowHeight="17205" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TUE FC Asset Plan SteerCo" sheetId="2" state="hidden" r:id="rId1"/>
@@ -154,7 +154,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1671" uniqueCount="656">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1682" uniqueCount="661">
   <si>
     <t>Fulfillment New Assets SteerCo (Tuesday's)</t>
   </si>
@@ -2411,6 +2411,21 @@
   </si>
   <si>
     <t xml:space="preserve">Advaith Venkataraman / Andrew </t>
+  </si>
+  <si>
+    <t>Not approved to move forward with Spec Building</t>
+  </si>
+  <si>
+    <t>26_01_29 Northeast Spec Bld Analysis.pptx</t>
+  </si>
+  <si>
+    <t>Adam Dunbar, Vik Gopalakrishnan, Jack Anderson, Jacob Shub</t>
+  </si>
+  <si>
+    <t>Spec Building Analysis for Northeast</t>
+  </si>
+  <si>
+    <t>26_05_08 SteerCo.pptx</t>
   </si>
 </sst>
 </file>
@@ -2547,7 +2562,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -2587,6 +2602,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2874,7 +2895,7 @@
     <xf numFmtId="44" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="15" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="144">
+  <cellXfs count="145">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3265,6 +3286,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="22" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -11802,7 +11826,7 @@
       </c>
       <c r="AI67" s="91"/>
     </row>
-    <row r="68" spans="1:35" s="32" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:35" s="32" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="33">
         <f>IF(ISBLANK(E68),"",_xlfn.XLOOKUP(E68,Info!A:A,Info!B:B))</f>
         <v>14</v>
@@ -11851,7 +11875,7 @@
       <c r="P68" s="92"/>
       <c r="AI68" s="91"/>
     </row>
-    <row r="69" spans="1:35" s="32" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:35" s="32" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="33">
         <f>IF(ISBLANK(E69),"",_xlfn.XLOOKUP(E69,Info!A:A,Info!B:B))</f>
         <v>14</v>
@@ -11941,6 +11965,9 @@
       <c r="L70" s="33"/>
       <c r="M70" s="67"/>
       <c r="N70" s="92"/>
+      <c r="O70" s="118" t="s">
+        <v>660</v>
+      </c>
       <c r="P70" s="92"/>
       <c r="AI70" s="91"/>
     </row>
@@ -12395,28 +12422,58 @@
       </c>
       <c r="AI80" s="91"/>
     </row>
-    <row r="81" spans="1:35" s="32" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="33" t="str">
+    <row r="81" spans="1:35" s="32" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A81" s="33" t="e">
         <f>IF(ISBLANK(E81),"",_xlfn.XLOOKUP(E81,Info!A:A,Info!B:B))</f>
-        <v/>
-      </c>
-      <c r="B81" s="33"/>
-      <c r="C81" s="33"/>
-      <c r="D81" s="54"/>
-      <c r="E81" s="91"/>
-      <c r="F81" s="54"/>
-      <c r="G81" s="33" t="str">
+        <v>#N/A</v>
+      </c>
+      <c r="B81" s="33" t="s">
+        <v>270</v>
+      </c>
+      <c r="C81" s="33" t="s">
+        <v>187</v>
+      </c>
+      <c r="D81" s="54" t="s">
+        <v>240</v>
+      </c>
+      <c r="E81" s="91">
+        <v>46051</v>
+      </c>
+      <c r="F81" s="54" t="s">
+        <v>659</v>
+      </c>
+      <c r="G81" s="33" t="e">
         <f>IF(ISBLANK(H81),"",_xlfn.XLOOKUP(H81,Info!A:A,Info!B:B))</f>
-        <v/>
-      </c>
-      <c r="H81" s="98"/>
-      <c r="I81" s="103"/>
-      <c r="J81" s="33"/>
-      <c r="K81" s="33"/>
-      <c r="L81" s="33"/>
-      <c r="M81" s="67"/>
-      <c r="N81" s="92"/>
-      <c r="P81" s="92"/>
+        <v>#N/A</v>
+      </c>
+      <c r="H81" s="98">
+        <f>E81-1</f>
+        <v>46050</v>
+      </c>
+      <c r="I81" s="103">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="J81" s="33">
+        <v>30</v>
+      </c>
+      <c r="K81" s="33" t="s">
+        <v>207</v>
+      </c>
+      <c r="L81" s="33" t="s">
+        <v>245</v>
+      </c>
+      <c r="M81" s="67" t="s">
+        <v>249</v>
+      </c>
+      <c r="N81" s="92" t="s">
+        <v>656</v>
+      </c>
+      <c r="O81" s="118" t="s">
+        <v>657</v>
+      </c>
+      <c r="P81" s="92" t="s">
+        <v>658</v>
+      </c>
       <c r="AI81" s="91"/>
     </row>
     <row r="82" spans="1:35" s="32" customFormat="1" x14ac:dyDescent="0.25">
@@ -20671,6 +20728,8 @@
     <hyperlink ref="O62" r:id="rId50" display="https://teams.wal-mart.com/:p:/r/sites/TechnologyandAutomation/Shared Documents/PMO/Fulfillment/NextGens/02. Presentations/01.  Steer Co Presentations/26_04_30 SteerCo.pptx?d=wdb87420320c440f3a352dd4f0e632eb9&amp;csf=1&amp;web=1&amp;e=B6iMdT" xr:uid="{6BF12395-B556-46A4-85ED-12F1DEAE5FDB}"/>
     <hyperlink ref="O61" r:id="rId51" display="https://teams.wal-mart.com/:p:/r/sites/TechnologyandAutomation/Shared Documents/PMO/Fulfillment/NextGens/02. Presentations/01.  Steer Co Presentations/26_04_30 SteerCo.pptx?d=wdb87420320c440f3a352dd4f0e632eb9&amp;csf=1&amp;web=1&amp;e=B6iMdT" xr:uid="{F70C6EE1-3B65-42A7-BDCF-59B2DC98581C}"/>
     <hyperlink ref="O68" r:id="rId52" display="https://teams.wal-mart.com/:p:/r/sites/TechnologyandAutomation/Shared Documents/PMO/Fulfillment/NextGens/02. Presentations/01.  Steer Co Presentations/26_05_04 SteerCo.pptx?d=wd44f71dddce1499cb3c5f8a6f9c7fd63&amp;csf=1&amp;web=1&amp;e=40F5If" xr:uid="{60F2AB70-8A56-4F25-B312-E392A4388BC6}"/>
+    <hyperlink ref="O81" r:id="rId53" display="https://teams.wal-mart.com/:p:/r/sites/TechnologyandAutomation/Shared Documents/PMO/Fulfillment/NextGens/02. Presentations/01.  Steer Co Presentations/26_01_29 Northeast Spec Bld Analysis.pptx?d=w9c538d8635b94c129ba00ea7eac27a0e&amp;csf=1&amp;web=1&amp;e=Cn3L1m" xr:uid="{4A6DDCAA-2AC4-4B9D-9AB3-D4FFDD8113C4}"/>
+    <hyperlink ref="O70" r:id="rId54" display="https://teams.wal-mart.com/:p:/r/sites/TechnologyandAutomation/Shared Documents/PMO/Fulfillment/NextGens/02. Presentations/01.  Steer Co Presentations/26_05_08 SteerCo.pptx?d=wd863957755e742f8bfaaadcb434b30d7&amp;csf=1&amp;web=1&amp;e=6FERxe" xr:uid="{A06FD16C-22D9-4F10-9FC7-D919C3472D73}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -21074,13 +21133,13 @@
       <c r="A16" s="97" t="s">
         <v>621</v>
       </c>
-      <c r="B16" s="98">
+      <c r="B16" s="144">
         <v>45859</v>
       </c>
-      <c r="C16" s="98">
+      <c r="C16" s="144">
         <v>46083</v>
       </c>
-      <c r="D16" s="98">
+      <c r="D16" s="144">
         <v>45992</v>
       </c>
       <c r="E16" s="98"/>
@@ -22283,7 +22342,7 @@
         <v>125</v>
       </c>
       <c r="D63" s="98">
-        <v>46170</v>
+        <v>46156</v>
       </c>
       <c r="E63" s="98" t="s">
         <v>125</v>
@@ -22475,21 +22534,21 @@
         <v>297</v>
       </c>
       <c r="N2" s="123">
-        <v>943000</v>
+        <v>643300</v>
       </c>
       <c r="O2" s="123">
-        <v>73205</v>
+        <v>432505</v>
       </c>
       <c r="P2" s="123">
         <v>144708</v>
       </c>
       <c r="Q2" s="123">
         <f>O2+P2</f>
-        <v>217913</v>
+        <v>577213</v>
       </c>
       <c r="R2" s="124">
         <f>Q2/N2</f>
-        <v>0.23108483563096502</v>
+        <v>0.89726877040261155</v>
       </c>
       <c r="S2" t="s">
         <v>497</v>
@@ -22652,7 +22711,7 @@
         <v>308</v>
       </c>
       <c r="N5" s="123">
-        <v>4700300</v>
+        <v>5000000</v>
       </c>
       <c r="O5" s="123">
         <v>1364948</v>
@@ -22666,7 +22725,7 @@
       </c>
       <c r="R5" s="124">
         <f>Q5/N5</f>
-        <v>0.75638789013467222</v>
+        <v>0.71104999999999996</v>
       </c>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.25">
@@ -26912,15 +26971,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E2EBBACD82105340A91324964E93FF49" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="7329edaaee89349510b5fe31ddec06b8">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a8552d75-6f1f-4d52-93a3-fcd36dc2752d" xmlns:ns3="1785dff3-9909-4165-bde0-36ec47a4b18f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="52e457d9bdc8fb3aec099fc7d60c5993" ns2:_="" ns3:_="">
     <xsd:import namespace="a8552d75-6f1f-4d52-93a3-fcd36dc2752d"/>
@@ -27155,6 +27205,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{752F9F6E-B88F-40CF-A00D-5A52044E6B25}">
   <ds:schemaRefs>
@@ -27173,14 +27232,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B8993D78-ABDB-48CF-A6AD-3E9555EB10CC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{89752E9E-F7C9-411F-9EA3-B9C1D8EEB123}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -27197,4 +27248,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B8993D78-ABDB-48CF-A6AD-3E9555EB10CC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>